<commit_message>
Infer store timezone from coordinates
</commit_message>
<xml_diff>
--- a/outputs/godaddy_prueba/admin/assets/layout_carga_tiendas.xlsx
+++ b/outputs/godaddy_prueba/admin/assets/layout_carga_tiendas.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tiendas'!$A$1:$G$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo zonas'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo zonas'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -200,7 +200,7 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Usa una clave: CENTRO, SONORA, PACIFICO, BAJA o CANCUN. Si se deja vacio, se tomara CENTRO.</t>
+        <t>Usa AUTO para calcular por coordenadas. Tambien puedes usar: CENTRO, SONORA, PACIFICO, BAJA o CANCUN.</t>
       </text>
     </comment>
   </commentList>
@@ -572,7 +572,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>SONORA</t>
+          <t>AUTO</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>AUTO</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>BAJA</t>
+          <t>AUTO</t>
         </is>
       </c>
     </row>
@@ -5132,8 +5132,8 @@
   </sheetData>
   <autoFilter ref="A1:G503"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G503" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Zona horaria invalida" error="Usa una clave valida del catalogo de zonas horarias." promptTitle="Zona horaria" prompt="Selecciona: CENTRO, SONORA, PACIFICO, BAJA o CANCUN" type="list">
-      <formula1>"CENTRO,SONORA,PACIFICO,BAJA,CANCUN"</formula1>
+    <dataValidation sqref="G2:G503" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Zona horaria invalida" error="Usa una clave valida del catalogo de zonas horarias." promptTitle="Zona horaria" prompt="Selecciona AUTO o una zona manual: CENTRO, SONORA, PACIFICO, BAJA o CANCUN" type="list">
+      <formula1>"AUTO,CENTRO,SONORA,PACIFICO,BAJA,CANCUN"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5147,7 +5147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5181,115 +5181,137 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Automatico por coordenadas</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Calculado por el sistema</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Recomendado para la carga masiva normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
           <t>CENTRO</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Centro / Monterrey / CDMX</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>America/Mexico_City</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>CDMX, Monterrey, Guadalajara, Puebla, Queretaro, Merida</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>SONORA</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Sonora / Hermosillo</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>America/Hermosillo</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Hermosillo y estado de Sonora</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>PACIFICO</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Pacifico / Sinaloa / BCS</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>America/Mazatlan</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Sinaloa, Culiacan, Mazatlan, La Paz, BCS</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>BAJA</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Baja California</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>America/Tijuana</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Tijuana, Mexicali, Baja California</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>CANCUN</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Quintana Roo / Cancun</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>America/Cancun</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Cancun y Quintana Roo</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>